<commit_message>
v1.0: four-company GHG dataset, SQL pipeline, Power BI report and README
</commit_message>
<xml_diff>
--- a/data/honda_raw.xlsx
+++ b/data/honda_raw.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ottob\Documents\Projects\Data Analytics\ghg-emissions-benchmarking\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D3272D-E972-4FE1-81F4-78BD136D97BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2B8CB2A-9375-4EC6-BA77-DC242962D0F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="34620" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -257,9 +257,6 @@
     <t>Not verified under limited assurance engagement for the year ended March 31, 2025.</t>
   </si>
   <si>
-    <t>Previous report aggregated this category under "Scope 3, other categories" — see Data Book 2024, p.150.</t>
-  </si>
-  <si>
     <t>Not restated — see Data Book 2024, p.150.</t>
   </si>
   <si>
@@ -267,9 +264,6 @@
 Not verified under limited assurance engagement for the year ended March 31, 2025.</t>
   </si>
   <si>
-    <t>Previous report aggregated this category under "Scope 3, other categories" — see Data Book 2023, p.138.</t>
-  </si>
-  <si>
     <t>Verified under limited assurance engagement for the year ended March 31, 2023 — see Data Book 2023, p.155. 
 Not verified under limited assurance engagement for the year ended March 31, 2025.</t>
   </si>
@@ -297,12 +291,6 @@
     <t>Not restated — see Data Book 2023, p.138.</t>
   </si>
   <si>
-    <t>Restated — see Data Book 2024, p.150: (267.39 million t-CO₂e).</t>
-  </si>
-  <si>
-    <t>Restated — see Data Book 2023, p.138: (284.41 million t-CO₂e).</t>
-  </si>
-  <si>
     <t>Only original value of Scope 3 Cat 11 verified under limited assurance engagement for the year ended March 31, 2024 — see Data Book 2024, p.166. 
 Current value not verified under limited assurance engagement for the year ended March 31, 2025.</t>
   </si>
@@ -326,20 +314,6 @@
   <si>
     <t>Not restated — see Data Book 2023, p.138. 
 Honda adopts the GHG Protocol’s standard market-based method — see ESG Report 2025, p.61.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">WORKBOOK: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>v1.0, 2026-10-16</t>
-    </r>
   </si>
   <si>
     <r>
@@ -728,6 +702,34 @@
   <si>
     <t>Global sales figures include motorcycles, automobiles and power products (power products: 381.2 ten thousand units) — see Honda Report 2024, p.5.
 Not republished in Honda Report 2025; value taken from the original report.</t>
+  </si>
+  <si>
+    <t>Restated — see Data Book 2024, p.150: (267.39 million t-CO₂e). 
+Honda changed the calculation of Categories 1, 4, 9 and 12 from the year ended March 31, 2025 and recalculated past performance — see ESG Report 2025, p.61.</t>
+  </si>
+  <si>
+    <t>First disclosed separately in ESG Report 2025; the earlier report included it only within “Scope 3, other categories”, so there is no original value to compare — see Data Book 2024, p.150.</t>
+  </si>
+  <si>
+    <t>First disclosed separately in ESG Report 2025; the earlier report included it only within “Scope 3, other categories”, so there is no original value to compare — see Data Book 2023, p.138.</t>
+  </si>
+  <si>
+    <t>Restated — see Data Book 2023, p.138: (284.41 million t-CO₂e). 
+Honda changed the calculation of Categories 1, 4, 9 and 12 from the year ended March 31, 2025 and recalculated past performance — see ESG Report 2025, p.61.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">WORKBOOK: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>v1.0, 2026-10-17</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1407,7 +1409,7 @@
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A1" s="10"/>
       <c r="B1" s="25" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C1" s="25"/>
       <c r="D1" s="25"/>
@@ -1416,7 +1418,7 @@
     <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10"/>
       <c r="B2" s="26" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C2" s="26"/>
       <c r="D2" s="26"/>
@@ -1425,7 +1427,7 @@
     <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="10"/>
       <c r="B3" s="26" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="C3" s="26"/>
       <c r="D3" s="26"/>
@@ -1434,7 +1436,7 @@
     <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10"/>
       <c r="B4" s="27" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C4" s="27"/>
       <c r="D4" s="27"/>
@@ -1457,7 +1459,7 @@
     <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="12"/>
       <c r="B7" s="14" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -1466,7 +1468,7 @@
     <row r="8" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="12"/>
       <c r="B8" s="20" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C8" s="20"/>
       <c r="D8" s="20"/>
@@ -1475,7 +1477,7 @@
     <row r="9" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="12"/>
       <c r="B9" s="20" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C9" s="20"/>
       <c r="D9" s="20"/>
@@ -1484,7 +1486,7 @@
     <row r="10" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="12"/>
       <c r="B10" s="20" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C10" s="20"/>
       <c r="D10" s="20"/>
@@ -1493,7 +1495,7 @@
     <row r="11" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="12"/>
       <c r="B11" s="20" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C11" s="20"/>
       <c r="D11" s="20"/>
@@ -1516,7 +1518,7 @@
     <row r="14" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="15"/>
       <c r="B14" s="17" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C14" s="15"/>
       <c r="D14" s="15"/>
@@ -1525,13 +1527,13 @@
     <row r="15" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="15"/>
       <c r="B15" s="16" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="E15" s="15"/>
     </row>
@@ -1541,36 +1543,36 @@
         <v>57</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="E16" s="15"/>
     </row>
     <row r="17" spans="1:5" ht="31" x14ac:dyDescent="0.35">
       <c r="A17" s="15"/>
       <c r="B17" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="C17" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="C17" s="19" t="s">
-        <v>114</v>
-      </c>
       <c r="D17" s="19" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E17" s="15"/>
     </row>
     <row r="18" spans="1:5" ht="31" x14ac:dyDescent="0.35">
       <c r="A18" s="15"/>
       <c r="B18" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="C18" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="C18" s="19" t="s">
-        <v>115</v>
-      </c>
       <c r="D18" s="19" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E18" s="15"/>
     </row>
@@ -1580,10 +1582,10 @@
         <v>60</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="E19" s="15"/>
     </row>
@@ -1593,10 +1595,10 @@
         <v>61</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E20" s="15"/>
     </row>
@@ -1606,10 +1608,10 @@
         <v>62</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E21" s="15"/>
     </row>
@@ -1630,7 +1632,7 @@
     <row r="24" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="15"/>
       <c r="B24" s="17" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C24" s="15"/>
       <c r="D24" s="15"/>
@@ -1639,7 +1641,7 @@
     <row r="25" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="15"/>
       <c r="B25" s="21" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="C25" s="22"/>
       <c r="D25" s="22"/>
@@ -1648,10 +1650,10 @@
     <row r="26" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="15"/>
       <c r="B26" s="18" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="C26" s="24" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="D26" s="24"/>
       <c r="E26" s="15"/>
@@ -1659,7 +1661,7 @@
     <row r="27" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="15"/>
       <c r="B27" s="23" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C27" s="23"/>
       <c r="D27" s="23"/>
@@ -1800,7 +1802,7 @@
         <v>58</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>59</v>
@@ -1899,7 +1901,7 @@
         <v>120</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="J2" s="3"/>
     </row>
@@ -1929,7 +1931,7 @@
         <v>120</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="J3" s="3"/>
     </row>
@@ -1959,7 +1961,7 @@
         <v>120</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="J4" s="3"/>
     </row>
@@ -2017,7 +2019,7 @@
         <v>91</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J6" s="3"/>
     </row>
@@ -2047,7 +2049,7 @@
         <v>91</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -2105,7 +2107,7 @@
         <v>91</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J9" s="3"/>
     </row>
@@ -2135,7 +2137,7 @@
         <v>91</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J10" s="3"/>
     </row>
@@ -2147,7 +2149,7 @@
         <v>45747</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D11" s="7">
         <v>2798.8</v>
@@ -2165,7 +2167,7 @@
         <v>7</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="J11" s="3"/>
     </row>
@@ -2177,7 +2179,7 @@
         <v>45382</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D12" s="7">
         <v>2674</v>
@@ -2195,7 +2197,7 @@
         <v>5</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="J12" s="3"/>
     </row>
@@ -2207,7 +2209,7 @@
         <v>45016</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D13" s="7">
         <v>2808.9</v>
@@ -2225,7 +2227,7 @@
         <v>3</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="J13" s="3"/>
     </row>
@@ -2362,10 +2364,10 @@
         <v>60</v>
       </c>
       <c r="K3" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="M3" s="3"/>
     </row>
@@ -2401,10 +2403,10 @@
         <v>60</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="M4" s="3"/>
     </row>
@@ -2440,7 +2442,7 @@
         <v>26</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
@@ -2477,7 +2479,7 @@
         <v>26</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
@@ -2514,7 +2516,7 @@
         <v>26</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
@@ -2551,7 +2553,7 @@
         <v>60</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="L8" s="3" t="s">
         <v>66</v>
@@ -2590,10 +2592,10 @@
         <v>60</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M9" s="3"/>
     </row>
@@ -2629,10 +2631,10 @@
         <v>60</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="M10" s="3"/>
     </row>
@@ -2705,10 +2707,10 @@
         <v>60</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>83</v>
+        <v>121</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="M12" s="3"/>
     </row>
@@ -2744,10 +2746,10 @@
         <v>60</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>84</v>
+        <v>124</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="M13" s="3"/>
     </row>
@@ -2891,7 +2893,7 @@
       </c>
       <c r="N2" s="3"/>
     </row>
-    <row r="3" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>58</v>
       </c>
@@ -2926,14 +2928,14 @@
         <v>60</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>70</v>
       </c>
       <c r="N3" s="3"/>
     </row>
-    <row r="4" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>58</v>
       </c>
@@ -2968,7 +2970,7 @@
         <v>60</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>70</v>
@@ -3015,7 +3017,7 @@
       </c>
       <c r="N5" s="3"/>
     </row>
-    <row r="6" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>58</v>
       </c>
@@ -3050,14 +3052,14 @@
         <v>60</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>70</v>
       </c>
       <c r="N6" s="3"/>
     </row>
-    <row r="7" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>58</v>
       </c>
@@ -3092,7 +3094,7 @@
         <v>60</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="M7" s="3" t="s">
         <v>70</v>
@@ -3139,7 +3141,7 @@
       </c>
       <c r="N8" s="3"/>
     </row>
-    <row r="9" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
         <v>58</v>
       </c>
@@ -3174,14 +3176,14 @@
         <v>60</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>70</v>
       </c>
       <c r="N9" s="3"/>
     </row>
-    <row r="10" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>58</v>
       </c>
@@ -3216,7 +3218,7 @@
         <v>60</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>70</v>
@@ -3263,7 +3265,7 @@
       </c>
       <c r="N11" s="3"/>
     </row>
-    <row r="12" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>58</v>
       </c>
@@ -3298,14 +3300,14 @@
         <v>60</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="M12" s="3" t="s">
         <v>70</v>
       </c>
       <c r="N12" s="3"/>
     </row>
-    <row r="13" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="3" t="s">
         <v>58</v>
       </c>
@@ -3340,7 +3342,7 @@
         <v>60</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="M13" s="3" t="s">
         <v>70</v>
@@ -3387,7 +3389,7 @@
       </c>
       <c r="N14" s="3"/>
     </row>
-    <row r="15" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>58</v>
       </c>
@@ -3422,14 +3424,14 @@
         <v>60</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="M15" s="3" t="s">
         <v>70</v>
       </c>
       <c r="N15" s="3"/>
     </row>
-    <row r="16" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="3" t="s">
         <v>58</v>
       </c>
@@ -3464,7 +3466,7 @@
         <v>60</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>70</v>
@@ -3511,7 +3513,7 @@
       </c>
       <c r="N17" s="3"/>
     </row>
-    <row r="18" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
         <v>58</v>
       </c>
@@ -3546,14 +3548,14 @@
         <v>60</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="M18" s="3" t="s">
         <v>70</v>
       </c>
       <c r="N18" s="3"/>
     </row>
-    <row r="19" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
         <v>58</v>
       </c>
@@ -3588,7 +3590,7 @@
         <v>60</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="M19" s="3" t="s">
         <v>70</v>
@@ -3635,7 +3637,7 @@
       </c>
       <c r="N20" s="3"/>
     </row>
-    <row r="21" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="3" t="s">
         <v>58</v>
       </c>
@@ -3670,14 +3672,14 @@
         <v>60</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>70</v>
       </c>
       <c r="N21" s="3"/>
     </row>
-    <row r="22" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
         <v>58</v>
       </c>
@@ -3712,7 +3714,7 @@
         <v>60</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="M22" s="3" t="s">
         <v>70</v>
@@ -3754,7 +3756,7 @@
         <v>26</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="M23" s="3"/>
       <c r="N23" s="3"/>
@@ -3794,7 +3796,7 @@
         <v>26</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="M24" s="3"/>
       <c r="N24" s="3"/>
@@ -3834,7 +3836,7 @@
         <v>26</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="M25" s="3"/>
       <c r="N25" s="3"/>
@@ -3879,7 +3881,7 @@
       </c>
       <c r="N26" s="3"/>
     </row>
-    <row r="27" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
         <v>58</v>
       </c>
@@ -3914,14 +3916,14 @@
         <v>60</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="M27" s="3" t="s">
         <v>70</v>
       </c>
       <c r="N27" s="3"/>
     </row>
-    <row r="28" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="3" t="s">
         <v>58</v>
       </c>
@@ -3956,7 +3958,7 @@
         <v>60</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="M28" s="3" t="s">
         <v>70</v>
@@ -4003,7 +4005,7 @@
       </c>
       <c r="N29" s="3"/>
     </row>
-    <row r="30" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="3" t="s">
         <v>58</v>
       </c>
@@ -4038,14 +4040,14 @@
         <v>60</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="M30" s="3" t="s">
         <v>70</v>
       </c>
       <c r="N30" s="3"/>
     </row>
-    <row r="31" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="3" t="s">
         <v>58</v>
       </c>
@@ -4080,7 +4082,7 @@
         <v>60</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="M31" s="3" t="s">
         <v>70</v>
@@ -4162,10 +4164,10 @@
         <v>60</v>
       </c>
       <c r="L33" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="M33" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="M33" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="N33" s="3"/>
     </row>
@@ -4204,10 +4206,10 @@
         <v>60</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="M34" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="N34" s="3"/>
     </row>
@@ -4251,7 +4253,7 @@
       </c>
       <c r="N35" s="3"/>
     </row>
-    <row r="36" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="3" t="s">
         <v>58</v>
       </c>
@@ -4286,14 +4288,14 @@
         <v>60</v>
       </c>
       <c r="L36" s="3" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="M36" s="3" t="s">
         <v>70</v>
       </c>
       <c r="N36" s="3"/>
     </row>
-    <row r="37" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="3" t="s">
         <v>58</v>
       </c>
@@ -4328,7 +4330,7 @@
         <v>60</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="M37" s="3" t="s">
         <v>70</v>
@@ -4370,7 +4372,7 @@
         <v>26</v>
       </c>
       <c r="L38" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="M38" s="3"/>
       <c r="N38" s="3"/>
@@ -4410,7 +4412,7 @@
         <v>26</v>
       </c>
       <c r="L39" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="M39" s="3"/>
       <c r="N39" s="3"/>
@@ -4450,7 +4452,7 @@
         <v>26</v>
       </c>
       <c r="L40" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="M40" s="3"/>
       <c r="N40" s="3"/>
@@ -4490,7 +4492,7 @@
         <v>26</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="M41" s="3"/>
       <c r="N41" s="3"/>
@@ -4530,7 +4532,7 @@
         <v>26</v>
       </c>
       <c r="L42" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="M42" s="3"/>
       <c r="N42" s="3"/>
@@ -4570,7 +4572,7 @@
         <v>26</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="M43" s="3"/>
       <c r="N43" s="3"/>
@@ -4615,7 +4617,7 @@
       </c>
       <c r="N44" s="3"/>
     </row>
-    <row r="45" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="3" t="s">
         <v>58</v>
       </c>
@@ -4650,14 +4652,14 @@
         <v>60</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="M45" s="3" t="s">
         <v>70</v>
       </c>
       <c r="N45" s="3"/>
     </row>
-    <row r="46" spans="1:14" ht="47.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:14" ht="78.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="3" t="s">
         <v>58</v>
       </c>
@@ -4692,7 +4694,7 @@
         <v>60</v>
       </c>
       <c r="L46" s="3" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="M46" s="3" t="s">
         <v>70</v>
@@ -4774,7 +4776,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">

</xml_diff>